<commit_message>
Add Labor-Leisure PDF and link it in Study Tracker Excel
- Create Labor_Leisure_Problems.pdf with all 6 LL problems (practice test Q3/Q4 + drills)
- Add source audit page noting no LL problems in uploaded HW/sample/lecture PDFs
- Link PDF in Study_Tracker.xlsx Practice Materials column for Labor-Leisure row
- Update Labor_Leisure_Problems.xlsx with PDF hyperlink

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Labor_Leisure_Problems.xlsx
+++ b/Labor_Leisure_Problems.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,11 +38,15 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="4">
@@ -89,11 +93,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -102,7 +108,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -471,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -496,178 +501,224 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Full PDF version (all problems + answer key):</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Labor_Leisure_Problems.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>Problem (solve on paper)</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Hints</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>Your work space</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="4" t="n">
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>LL-1 (Practice Test Q3)</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>All 3 practice tests — Q3</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>Maria has 16 hours/day for leisure (ℓ) and work. Wage w = $20/hr, non-labor income V = $80. Utility U(c, ℓ) = c^0.5 ℓ^0.5 where c = w(16 − ℓ) + V.
 Find: (a) optimal leisure ℓ*, (b) labor hours L*, (c) consumption c*.</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>Budget: c = w(16−ℓ)+V. Optimum: MU_ℓ/MU_c = w. Cobb-Douglas α=β=0.5 → c = wℓ.</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr"/>
-    </row>
-    <row r="6" ht="70" customHeight="1">
-      <c r="A6" s="4" t="n">
+      <c r="F6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7" ht="70" customHeight="1">
+      <c r="A7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>LL-2 (Practice Test Q4)</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>All 3 practice tests — Q4</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>Same setup as LL-1, but wage rises to w = $30/hr.
 Find: (a) new ℓ*, (b) new L*, (c) new c*. Does Maria work more or less than when w = $20?</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>Use ℓ* = (w·T + V) / (2w) with T = 16. Compare L* to LL-1.</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr"/>
-    </row>
-    <row r="7" ht="70" customHeight="1">
-      <c r="A7" s="4" t="n">
+      <c r="F7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8" ht="70" customHeight="1">
+      <c r="A8" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>LL-3</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Extra practice (study sheet)</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>Alex has 8 hours/day (T = 8). Wage w = $25/hr, V = $0. U(c, ℓ) = c^0.5 ℓ^0.5, c = w(8 − ℓ) + V.
 Find ℓ*, L*, and c*.</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>ℓ* = (wT + V)/(2w) when α = β = 0.5.</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr"/>
-    </row>
-    <row r="8" ht="70" customHeight="1">
-      <c r="A8" s="4" t="n">
+      <c r="F8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9" ht="70" customHeight="1">
+      <c r="A9" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>LL-4</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>Extra practice (study sheet)</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>Same as LL-3 but V = $40 (lottery winnings). w = $25, T = 8.
 Find ℓ*, L*, c*. Did leisure increase vs LL-3?</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>Higher V shifts budget outward → more leisure for Cobb-Douglas.</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr"/>
-    </row>
-    <row r="9" ht="70" customHeight="1">
-      <c r="A9" s="4" t="n">
+      <c r="F9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10" ht="70" customHeight="1">
+      <c r="A10" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>LL-5</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Extra practice (study sheet)</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>Jordan: T = 24 hrs, w = $15/hr, V = $60, U(c, ℓ) = c^0.25 ℓ^0.75 (loves leisure more than Maria).
 Find ℓ* using MU_ℓ/MU_c = w.</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>MRS = (0.75/0.25)(c/ℓ) = 3c/ℓ = w → c = (w/3)ℓ. Plug into budget.</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr"/>
+      <c r="F10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11" ht="70" customHeight="1">
+      <c r="A11" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>LL-6</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Extra practice (study sheet)</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Sam: T = 10 hrs, V = $100, U(c, ℓ) = c^0.5 ℓ^0.5.
+(a) w = $10: find ℓ*, L*
+(b) w = $40: find ℓ*, L*
+(c) As wage rises, work more or less?</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>ℓ* = (wT+V)/(2w). Compare L* = T − ℓ*.</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A3:B3"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="C3:F3"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -678,7 +729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -694,104 +745,121 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Bank ID</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>Answer / Solution sketch</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>LL-1 (Practice Test Q3)</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Q021</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>ℓ* = 10 hrs, L* = 6 hrs, c* = $200</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>LL-2 (Practice Test Q4)</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Q022</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>ℓ* ≈ 9.33 hrs, L* ≈ 6.67 hrs, c* ≈ $360. Works MORE.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>LL-3</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>ℓ* = 4 hrs, L* = 4 hrs, c* = $100</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>LL-4</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>ℓ* = 4.8 hrs, L* = 3.2 hrs, c* = $120. Yes — more leisure.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>LL-5</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>ℓ* ≈ 15.5 hrs, L* ≈ 8.5 hrs, c* ≈ $187.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>LL-6</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>(a) ℓ*=6, L*=4  (b) ℓ*=7.5, L*=2.5  (c) Works LESS</t>
         </is>
       </c>
     </row>
@@ -821,72 +889,72 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Setup</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>T = total hours, ℓ = leisure, L = labor hours, L = T − ℓ</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>c = w·L + V = w(T − ℓ) + V</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Optimum</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>MU_ℓ / MU_c = w  (MRS = wage)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Cobb-Douglas U = c^α ℓ^β</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>At optimum: β·c = α·w·ℓ</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Cobb-Douglas α = β = 0.5</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>c = w·ℓ  and  ℓ* = (w·T + V) / (2w)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Consumption</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>c* = w·ℓ* + V  (or w·L* + V)</t>
         </is>

</xml_diff>

<commit_message>
Fix Labor-Leisure PDF garbled symbols (use DejaVu font + ASCII notation)
Helvetica could not render leisure symbol and math punctuation, showing dots
instead. Switch to DejaVu Sans and use plain l for leisure, * for multiply.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Labor_Leisure_Problems.xlsx
+++ b/Labor_Leisure_Problems.xlsx
@@ -561,13 +561,13 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Maria has 16 hours/day for leisure (ℓ) and work. Wage w = $20/hr, non-labor income V = $80. Utility U(c, ℓ) = c^0.5 ℓ^0.5 where c = w(16 − ℓ) + V.
-Find: (a) optimal leisure ℓ*, (b) labor hours L*, (c) consumption c*.</t>
+          <t>Maria has 16 hours/day for leisure (l) and work. Wage w = $20/hr, non-labor income V = $80. Utility U(c, l) = c^0.5 * l^0.5 where c = w*(16 - l) + V.
+Find: (a) optimal leisure l*, (b) labor hours L*, (c) consumption c*.</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Budget: c = w(16−ℓ)+V. Optimum: MU_ℓ/MU_c = w. Cobb-Douglas α=β=0.5 → c = wℓ.</t>
+          <t>Budget: c = w*(16-l)+V. Optimum: MU_l/MU_c = w. Cobb-Douglas a=b=0.5 -&gt; c = w*l.</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr"/>
@@ -589,12 +589,12 @@
       <c r="D7" s="6" t="inlineStr">
         <is>
           <t>Same setup as LL-1, but wage rises to w = $30/hr.
-Find: (a) new ℓ*, (b) new L*, (c) new c*. Does Maria work more or less than when w = $20?</t>
+Find: (a) new l*, (b) new L*, (c) new c*. Does Maria work more or less than when w = $20?</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Use ℓ* = (w·T + V) / (2w) with T = 16. Compare L* to LL-1.</t>
+          <t>Use l* = (w*T + V) / (2w) with T = 16. Compare L* to LL-1.</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr"/>
@@ -615,13 +615,13 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Alex has 8 hours/day (T = 8). Wage w = $25/hr, V = $0. U(c, ℓ) = c^0.5 ℓ^0.5, c = w(8 − ℓ) + V.
-Find ℓ*, L*, and c*.</t>
+          <t>Alex has 8 hours/day (T = 8). Wage w = $25/hr, V = $0. U(c, l) = c^0.5 * l^0.5, c = w*(8 - l) + V.
+Find l*, L*, and c*.</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>ℓ* = (wT + V)/(2w) when α = β = 0.5.</t>
+          <t>l* = (w*T + V)/(2w) when a = b = 0.5.</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr"/>
@@ -643,12 +643,12 @@
       <c r="D9" s="6" t="inlineStr">
         <is>
           <t>Same as LL-3 but V = $40 (lottery winnings). w = $25, T = 8.
-Find ℓ*, L*, c*. Did leisure increase vs LL-3?</t>
+Find l*, L*, c*. Did leisure increase vs LL-3?</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Higher V shifts budget outward → more leisure for Cobb-Douglas.</t>
+          <t>Higher V shifts budget outward -&gt; more leisure for Cobb-Douglas.</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr"/>
@@ -669,13 +669,13 @@
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>Jordan: T = 24 hrs, w = $15/hr, V = $60, U(c, ℓ) = c^0.25 ℓ^0.75 (loves leisure more than Maria).
-Find ℓ* using MU_ℓ/MU_c = w.</t>
+          <t>Jordan: T = 24 hrs, w = $15/hr, V = $60, U(c, l) = c^0.25 * l^0.75 (loves leisure more than Maria).
+Find l* using MU_l/MU_c = w.</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>MRS = (0.75/0.25)(c/ℓ) = 3c/ℓ = w → c = (w/3)ℓ. Plug into budget.</t>
+          <t>MRS = (0.75/0.25)*(c/l) = 3c/l = w -&gt; c = (w/3)*l. Plug into budget.</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr"/>
@@ -696,15 +696,15 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Sam: T = 10 hrs, V = $100, U(c, ℓ) = c^0.5 ℓ^0.5.
-(a) w = $10: find ℓ*, L*
-(b) w = $40: find ℓ*, L*
+          <t>Sam: T = 10 hrs, V = $100, U(c, l) = c^0.5 * l^0.5.
+(a) w = $10: find l*, L*
+(b) w = $40: find l*, L*
 (c) As wage rises, work more or less?</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>ℓ* = (wT+V)/(2w). Compare L* = T − ℓ*.</t>
+          <t>l* = (w*T+V)/(2w). Compare L* = T - l*.</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr"/>
@@ -774,7 +774,7 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>ℓ* = 10 hrs, L* = 6 hrs, c* = $200</t>
+          <t>l* = 10 hrs, L* = 6 hrs, c* = $200</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>ℓ* ≈ 9.33 hrs, L* ≈ 6.67 hrs, c* ≈ $360. Works MORE.</t>
+          <t>l* = 9.33 hrs, L* = 6.67 hrs, c* = $360. Works MORE.</t>
         </is>
       </c>
     </row>
@@ -808,7 +808,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>ℓ* = 4 hrs, L* = 4 hrs, c* = $100</t>
+          <t>l* = 4 hrs, L* = 4 hrs, c* = $100</t>
         </is>
       </c>
     </row>
@@ -825,7 +825,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>ℓ* = 4.8 hrs, L* = 3.2 hrs, c* = $120. Yes — more leisure.</t>
+          <t>l* = 4.8 hrs, L* = 3.2 hrs, c* = $120. Yes - more leisure.</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>ℓ* ≈ 15.5 hrs, L* ≈ 8.5 hrs, c* ≈ $187.50</t>
+          <t>l* = 15.5 hrs, L* = 8.5 hrs, c* = $187.50</t>
         </is>
       </c>
     </row>
@@ -859,7 +859,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>(a) ℓ*=6, L*=4  (b) ℓ*=7.5, L*=2.5  (c) Works LESS</t>
+          <t>(a) l*=6, L*=4  (b) l*=7.5, L*=2.5  (c) Works LESS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Embed Labor-Leisure PDF inside Excel workbooks
- Add PDF tab with all 9 pages as images for viewing in Excel
- Package raw PDF inside xlsx (xl/embeddings/)
- Study Tracker Labor-Leisure row links to embedded PDF tab

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Labor_Leisure_Problems.xlsx
+++ b/Labor_Leisure_Problems.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Problems to Solve" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Answer Key" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formula Sheet" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PDF" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Problems to Solve" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Answer Key" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formula Sheet" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,6 +48,10 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="4">
@@ -93,8 +98,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -185,6 +191,236 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="8867775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>64</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="8867775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>128</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="8867775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>192</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="8867775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>255</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="8867775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>319</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="8867775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>383</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="8867775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>446</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="8867775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>510</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="8867775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -476,6 +712,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="105" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Full PDF below (same as Labor_Leisure_Problems.pdf)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -488,213 +749,213 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Labor-Leisure Problems — ECON 351</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>The uploaded file 'Econ351Lecture_2__Chapter_9___2__ea6a.pdf' is Chapter 9 (Uncertainty &amp; Risk) only. It contains NO labor-leisure problems. Labor-leisure is Chapter 4 consumer theory.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Full PDF version (all problems + answer key):</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Labor_Leisure_Problems.pdf</t>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Full PDF (included in this workbook — see 'PDF' tab):</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Open online copy</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>Problem (solve on paper)</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>Hints</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>Your work space</t>
         </is>
       </c>
     </row>
     <row r="6" ht="80" customHeight="1">
-      <c r="A6" s="6" t="n">
+      <c r="A6" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>LL-1 (Practice Test Q3)</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>All 3 practice tests — Q3</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>Maria has 16 hours/day for leisure (l) and work. Wage w = $20/hr, non-labor income V = $80. Utility U(c, l) = c^0.5 * l^0.5 where c = w*(16 - l) + V.
 Find: (a) optimal leisure l*, (b) labor hours L*, (c) consumption c*.</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>Budget: c = w*(16-l)+V. Optimum: MU_l/MU_c = w. Cobb-Douglas a=b=0.5 -&gt; c = w*l.</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
     </row>
     <row r="7" ht="70" customHeight="1">
-      <c r="A7" s="6" t="n">
+      <c r="A7" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>LL-2 (Practice Test Q4)</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>All 3 practice tests — Q4</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>Same setup as LL-1, but wage rises to w = $30/hr.
 Find: (a) new l*, (b) new L*, (c) new c*. Does Maria work more or less than when w = $20?</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>Use l* = (w*T + V) / (2w) with T = 16. Compare L* to LL-1.</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
     </row>
     <row r="8" ht="70" customHeight="1">
-      <c r="A8" s="6" t="n">
+      <c r="A8" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>LL-3</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>Extra practice (study sheet)</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>Alex has 8 hours/day (T = 8). Wage w = $25/hr, V = $0. U(c, l) = c^0.5 * l^0.5, c = w*(8 - l) + V.
 Find l*, L*, and c*.</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>l* = (w*T + V)/(2w) when a = b = 0.5.</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr"/>
+      <c r="F8" s="7" t="inlineStr"/>
     </row>
     <row r="9" ht="70" customHeight="1">
-      <c r="A9" s="6" t="n">
+      <c r="A9" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>LL-4</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Extra practice (study sheet)</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>Same as LL-3 but V = $40 (lottery winnings). w = $25, T = 8.
 Find l*, L*, c*. Did leisure increase vs LL-3?</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>Higher V shifts budget outward -&gt; more leisure for Cobb-Douglas.</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr"/>
+      <c r="F9" s="7" t="inlineStr"/>
     </row>
     <row r="10" ht="70" customHeight="1">
-      <c r="A10" s="6" t="n">
+      <c r="A10" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>LL-5</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>Extra practice (study sheet)</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>Jordan: T = 24 hrs, w = $15/hr, V = $60, U(c, l) = c^0.25 * l^0.75 (loves leisure more than Maria).
 Find l* using MU_l/MU_c = w.</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>MRS = (0.75/0.25)*(c/l) = 3c/l = w -&gt; c = (w/3)*l. Plug into budget.</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr"/>
+      <c r="F10" s="7" t="inlineStr"/>
     </row>
     <row r="11" ht="70" customHeight="1">
-      <c r="A11" s="6" t="n">
+      <c r="A11" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>LL-6</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>Extra practice (study sheet)</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>Sam: T = 10 hrs, V = $100, U(c, l) = c^0.5 * l^0.5.
 (a) w = $10: find l*, L*
@@ -702,12 +963,12 @@
 (c) As wage rises, work more or less?</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>l* = (w*T+V)/(2w). Compare L* = T - l*.</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr"/>
+      <c r="F11" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -723,7 +984,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -738,126 +999,126 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Answer Key — Labor-Leisure</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Bank ID</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>Answer / Solution sketch</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>LL-1 (Practice Test Q3)</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>Q021</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>l* = 10 hrs, L* = 6 hrs, c* = $200</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>LL-2 (Practice Test Q4)</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Q022</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>l* = 9.33 hrs, L* = 6.67 hrs, c* = $360. Works MORE.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>LL-3</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>l* = 4 hrs, L* = 4 hrs, c* = $100</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>LL-4</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>l* = 4.8 hrs, L* = 3.2 hrs, c* = $120. Yes - more leisure.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>LL-5</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>l* = 15.5 hrs, L* = 8.5 hrs, c* = $187.50</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>LL-6</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>(a) l*=6, L*=4  (b) l*=7.5, L*=2.5  (c) Works LESS</t>
         </is>
@@ -868,7 +1129,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -882,81 +1143,81 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Labor-Leisure Formula Sheet</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Setup</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>T = total hours, ℓ = leisure, L = labor hours, L = T − ℓ</t>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>T = total hours, l = leisure, L = labor hours, L = T - l</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>c = w·L + V = w(T − ℓ) + V</t>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>c = w*L + V = w*(T - l) + V</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Optimum</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>MU_ℓ / MU_c = w  (MRS = wage)</t>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>MU_l / MU_c = w  (MRS = wage)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Cobb-Douglas U = c^α ℓ^β</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>At optimum: β·c = α·w·ℓ</t>
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Cobb-Douglas U = c^a * l^b</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>At optimum: b*c = a*w*l</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Cobb-Douglas α = β = 0.5</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>c = w·ℓ  and  ℓ* = (w·T + V) / (2w)</t>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Cobb-Douglas a = b = 0.5</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>c = w*l  and  l* = (w*T + V) / (2w)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Consumption</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>c* = w·ℓ* + V  (or w·L* + V)</t>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>c* = w*l* + V  (or w*L* + V)</t>
         </is>
       </c>
     </row>

</xml_diff>